<commit_message>
fix date in HMPV
</commit_message>
<xml_diff>
--- a/example_files/HMPV_metadata_template.xlsx
+++ b/example_files/HMPV_metadata_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10920"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85A85FC2-5278-2B42-BEB2-C5EA54F7C5BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC93E528-87AC-FD41-91C4-9BE29961E494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14100" yWindow="-22380" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1607,7 +1607,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="872">
   <si>
     <t>id</t>
   </si>
@@ -4217,9 +4217,6 @@
   </si>
   <si>
     <t>Homo sapiens</t>
-  </si>
-  <si>
-    <t>15/06/2023</t>
   </si>
   <si>
     <t>USA/WA-UW-1b519/2023</t>
@@ -4302,7 +4299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -4320,8 +4317,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5002,19 +4998,19 @@
       </c>
     </row>
     <row r="2" spans="1:86" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" t="s">
         <v>861</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" t="s">
         <v>519</v>
       </c>
-      <c r="C2" s="14" t="s">
-        <v>870</v>
-      </c>
-      <c r="D2" s="13" t="s">
+      <c r="C2" s="13">
+        <v>45092</v>
+      </c>
+      <c r="D2" t="s">
         <v>865</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" t="s">
         <v>863</v>
       </c>
       <c r="F2" t="s">
@@ -5027,23 +5023,23 @@
         <v>868</v>
       </c>
       <c r="Q2" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="3" spans="1:86" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="13" t="s">
+      <c r="A3" t="s">
         <v>862</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" t="s">
         <v>368</v>
       </c>
-      <c r="C3" s="15">
+      <c r="C3" s="14">
         <v>45576</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" t="s">
         <v>866</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" t="s">
         <v>864</v>
       </c>
       <c r="F3" t="s">
@@ -5053,7 +5049,7 @@
         <v>868</v>
       </c>
       <c r="Q3" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
   </sheetData>

</xml_diff>